<commit_message>
Ingest technology, anglofuturism and full-stack themes
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CD5E06-0D0F-488D-A449-2AEF2D0FD2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A7015E-3015-4E6B-8D8B-5F3003B9B048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="249">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -608,6 +608,177 @@
   </si>
   <si>
     <t>Elite Theory &amp; Cyclical History</t>
+  </si>
+  <si>
+    <t>technoloogy</t>
+  </si>
+  <si>
+    <t>Advanced Technology</t>
+  </si>
+  <si>
+    <t>anglofuturism</t>
+  </si>
+  <si>
+    <t>full-stack</t>
+  </si>
+  <si>
+    <t>The Full Stack</t>
+  </si>
+  <si>
+    <t>Anglofutrism</t>
+  </si>
+  <si>
+    <t>Not possible British Futures…destiny.</t>
+  </si>
+  <si>
+    <t>Grounded but hyper-ambitious</t>
+  </si>
+  <si>
+    <t>No Anglofuturism without the Future</t>
+  </si>
+  <si>
+    <t>Britain dreams of itself</t>
+  </si>
+  <si>
+    <t>Recommendations, not endorsements</t>
+  </si>
+  <si>
+    <t>A deep idea of time, place and meaning</t>
+  </si>
+  <si>
+    <t>Demis Hassabis, Mustafa Suleyman, Geoffrey Hinton</t>
+  </si>
+  <si>
+    <t>Foundational resources of Anglofuturism</t>
+  </si>
+  <si>
+    <t>Aris Roussinos, Alexander D’Albini, Tom Ough,  Tom Ough, Calum Drysdale, Aeron Laffere</t>
+  </si>
+  <si>
+    <t>Substack for those ordained and yet to be ordained as Anglofuturists</t>
+  </si>
+  <si>
+    <t>Ideas matter A LOT to Anglofuturism</t>
+  </si>
+  <si>
+    <t>Roots &amp; Wings</t>
+  </si>
+  <si>
+    <t>Frank Furedi</t>
+  </si>
+  <si>
+    <t>Contra Western decline</t>
+  </si>
+  <si>
+    <t>Alasdair's Substack</t>
+  </si>
+  <si>
+    <t>Alasdair J. Marshall</t>
+  </si>
+  <si>
+    <t>institutional and political reform</t>
+  </si>
+  <si>
+    <t>Domesday Foundation</t>
+  </si>
+  <si>
+    <t>https://domesdayfoundation.substack.com/</t>
+  </si>
+  <si>
+    <t>Building the next regime.</t>
+  </si>
+  <si>
+    <t>Doomsday Foundation</t>
+  </si>
+  <si>
+    <t>https://alasdairjmarshall.substack.com/</t>
+  </si>
+  <si>
+    <t>https://frankfuredi.substack.com/</t>
+  </si>
+  <si>
+    <t>https://www.academyofideas.uk/</t>
+  </si>
+  <si>
+    <t>Academy of Ideas</t>
+  </si>
+  <si>
+    <t>When we said ideas matter, we meant it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ready </t>
+  </si>
+  <si>
+    <t>technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Substack </t>
+  </si>
+  <si>
+    <t>Planetocracy</t>
+  </si>
+  <si>
+    <t>Peter Hague</t>
+  </si>
+  <si>
+    <t>https://planetocracy.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Our future in space</t>
+  </si>
+  <si>
+    <t>https://anglofuturismblast.substack.com/</t>
+  </si>
+  <si>
+    <t>All Things Anglofuturist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anglofuturism Blast </t>
+  </si>
+  <si>
+    <t>Alexander D’Albini</t>
+  </si>
+  <si>
+    <t>podcast</t>
+  </si>
+  <si>
+    <t>Anglofuturism Podcast</t>
+  </si>
+  <si>
+    <t>Tom Ough, Callum Drysdale</t>
+  </si>
+  <si>
+    <t>https://podcasts.apple.com/gb/podcast/anglofuturism/id1743404902</t>
+  </si>
+  <si>
+    <t>The Future of Britain</t>
+  </si>
+  <si>
+    <t>free</t>
+  </si>
+  <si>
+    <t>Analytical and always on point</t>
+  </si>
+  <si>
+    <t>New thinking, new ideas</t>
+  </si>
+  <si>
+    <t>A possible branching future</t>
+  </si>
+  <si>
+    <t>The ideas factory</t>
+  </si>
+  <si>
+    <t>Space exploration, British style</t>
+  </si>
+  <si>
+    <t>One of the originators</t>
+  </si>
+  <si>
+    <t>Popularizers of Anglofuturism</t>
+  </si>
+  <si>
+    <t>Multiple thinkers, Multiple ideas</t>
   </si>
 </sst>
 </file>
@@ -750,15 +921,15 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1073,16 +1244,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
+      <c r="B1" s="12"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11"/>
+      <c r="B3" s="12"/>
     </row>
     <row r="5" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1200,44 +1371,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
     </row>
     <row r="2" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
     </row>
     <row r="3" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1453,7 +1624,7 @@
       <c r="B9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>152</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -1462,7 +1633,7 @@
       <c r="E9" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="10" t="s">
         <v>171</v>
       </c>
       <c r="G9" s="6" t="s">
@@ -2185,34 +2356,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
     </row>
     <row r="3" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2350,69 +2521,123 @@
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>166</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="10" t="s">
         <v>169</v>
       </c>
       <c r="I8" s="6">
         <v>7</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="10" t="s">
         <v>49</v>
       </c>
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
+      <c r="B9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="I9" s="6">
+        <v>6</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
+      <c r="B10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10" s="6">
+        <v>5</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="I11" s="6">
+        <v>4</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -2886,38 +3111,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
     </row>
     <row r="2" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
     </row>
     <row r="3" spans="1:13" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -3005,7 +3230,7 @@
       <c r="B6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="10" t="s">
         <v>166</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -3023,7 +3248,7 @@
       <c r="H6" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="10" t="s">
         <v>173</v>
       </c>
       <c r="J6" s="6">
@@ -3032,7 +3257,7 @@
       <c r="K6" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="L6" s="14" t="s">
+      <c r="L6" s="10" t="s">
         <v>49</v>
       </c>
       <c r="M6" s="6"/>
@@ -3042,7 +3267,7 @@
       <c r="B7" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>166</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -3051,7 +3276,7 @@
       <c r="E7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="10" t="s">
         <v>178</v>
       </c>
       <c r="G7" s="6" t="s">
@@ -3060,7 +3285,7 @@
       <c r="H7" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="10" t="s">
         <v>181</v>
       </c>
       <c r="J7" s="6">
@@ -3069,7 +3294,7 @@
       <c r="K7" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="L7" s="14" t="s">
+      <c r="L7" s="10" t="s">
         <v>49</v>
       </c>
       <c r="M7" s="6"/>
@@ -3079,7 +3304,7 @@
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>123</v>
       </c>
       <c r="D8" s="6" t="s">
@@ -3088,16 +3313,16 @@
       <c r="E8" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="10" t="s">
         <v>183</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="I8" s="14" t="s">
+      <c r="I8" s="10" t="s">
         <v>186</v>
       </c>
       <c r="J8" s="6">
@@ -3106,7 +3331,7 @@
       <c r="K8" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="L8" s="14" t="s">
+      <c r="L8" s="10" t="s">
         <v>49</v>
       </c>
       <c r="M8" s="6"/>
@@ -3116,25 +3341,25 @@
       <c r="B9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>128</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="10" t="s">
         <v>188</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="10" t="s">
         <v>191</v>
       </c>
       <c r="J9" s="6">
@@ -3143,114 +3368,268 @@
       <c r="K9" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="L9" s="14" t="s">
+      <c r="L9" s="10" t="s">
         <v>49</v>
       </c>
       <c r="M9" s="6"/>
     </row>
     <row r="10" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
+      <c r="B10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="J10" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M10" s="6"/>
     </row>
     <row r="11" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="J11" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M11" s="6"/>
     </row>
     <row r="12" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="J12" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M12" s="6"/>
     </row>
     <row r="13" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
+      <c r="B13" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J13" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M13" s="6"/>
     </row>
     <row r="14" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
+      <c r="B14" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="J14" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M14" s="6"/>
     </row>
     <row r="15" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
+      <c r="B15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="J15" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M15" s="6"/>
     </row>
     <row r="16" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
+      <c r="B16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="J16" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M16" s="6"/>
     </row>
     <row r="17" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3692,6 +4071,9 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="G6" r:id="rId1" xr:uid="{383BF627-0112-41D4-9CE5-464558D56F8E}"/>
+    <hyperlink ref="G10" r:id="rId2" xr:uid="{DFC55BEA-AE38-403E-9278-B5F569C5550E}"/>
+    <hyperlink ref="G14" r:id="rId3" xr:uid="{2A49FE45-E390-45E3-8D17-85E446CE2E31}"/>
+    <hyperlink ref="G16" r:id="rId4" xr:uid="{D7BAF8CC-72B4-428E-A765-C89F97972091}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -3718,22 +4100,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -3909,22 +4291,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Ingest intercepts dead-drop; refresh thinkers constellation
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A7015E-3015-4E6B-8D8B-5F3003B9B048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9954A2F8-9269-4B9D-A92E-B09C305AF7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,10 @@
     <sheet name="RESOURCES" sheetId="4" r:id="rId4"/>
     <sheet name="JOIN_ROADMAP" sheetId="5" r:id="rId5"/>
     <sheet name="PAGES" sheetId="6" r:id="rId6"/>
+    <sheet name="INTERCEPTS" sheetId="12" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">INTERCEPTS!$A$4:$N$200</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">JOIN_ROADMAP!$A$4:$E$200</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">PAGES!$A$4:$E$200</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">RESOURCES!$A$4:$M$200</definedName>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="286">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -511,15 +513,9 @@
     <t>Visionary</t>
   </si>
   <si>
-    <t>Sam Bowman</t>
-  </si>
-  <si>
     <t>Articulates the materialist, supply-side backbone of British techno-optimism.</t>
   </si>
   <si>
-    <t>Makes an Anglofuturist vision physically viable.</t>
-  </si>
-  <si>
     <t>https://worksinprogress.co/</t>
   </si>
   <si>
@@ -779,13 +775,130 @@
   </si>
   <si>
     <t>Multiple thinkers, Multiple ideas</t>
+  </si>
+  <si>
+    <t>Logos Movement</t>
+  </si>
+  <si>
+    <t>The embodiment of refusing the envelope - alternative futures are available.</t>
+  </si>
+  <si>
+    <t>Builders</t>
+  </si>
+  <si>
+    <t>https://logos.co/</t>
+  </si>
+  <si>
+    <t>Exemplar not script</t>
+  </si>
+  <si>
+    <t>Works in Progress</t>
+  </si>
+  <si>
+    <t>Futurism, Habitation, Infrastructure</t>
+  </si>
+  <si>
+    <t>Privacy-first movement that builds decentralized technology and local civic communities to establish a parallel, self-reliant society free from centralized surveillance and corporate control.</t>
+  </si>
+  <si>
+    <t>Suppliers of competence and know-how.</t>
+  </si>
+  <si>
+    <t>Thinkers</t>
+  </si>
+  <si>
+    <t>John Ruskin</t>
+  </si>
+  <si>
+    <t>Championed a return to craft, hierarchy, and producer guilds</t>
+  </si>
+  <si>
+    <t>https://www.guildofstgeorge.org.uk/resources/readings-from-ruskin</t>
+  </si>
+  <si>
+    <t>Governance, Craft</t>
+  </si>
+  <si>
+    <t>Borrow the Aesthetics and convinctions only.</t>
+  </si>
+  <si>
+    <t>Provides Anglofuturismss core moral aesthetic: the conviction that an authentic future cannot be built on soulless mass-fabrication, but must instead fuse native vernacular craft, organic materials, and human-scale dignity with advanced technological capability.</t>
+  </si>
+  <si>
+    <t>show_from</t>
+  </si>
+  <si>
+    <t>show_until</t>
+  </si>
+  <si>
+    <t>then_file_as</t>
+  </si>
+  <si>
+    <t>2026-10-13</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>Public conversation. Not a party broadcast.</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>Import this sheet into the catalog workbook (or File &gt; Import in Google Sheets). Max 3 ready rows with show_from ≤ today ≤ show_until appear on the homepage. Leave id blank.</t>
+  </si>
+  <si>
+    <t>INTERCEPTS — this week's dead-drop</t>
+  </si>
+  <si>
+    <t>AI doom and Britain’s factory boom</t>
+  </si>
+  <si>
+    <t>https://podcasts.apple.com/gb/podcast/ai-doom-and-britains-factory-boom/id1743404902?i=1000791082984</t>
+  </si>
+  <si>
+    <t>Latest AF podcast intercept</t>
+  </si>
+  <si>
+    <t>https://forbiddentexts.substack.com/p/on-elite-theory-clearing-up-conceptual</t>
+  </si>
+  <si>
+    <t>On Elite Theory: Clearing Up Conceptual Confusion, An FAQ</t>
+  </si>
+  <si>
+    <t>essay</t>
+  </si>
+  <si>
+    <t>Neema Parvini Substack</t>
+  </si>
+  <si>
+    <t>Concise primer on Elite theory</t>
+  </si>
+  <si>
+    <t>drop</t>
+  </si>
+  <si>
+    <t>https://frankfuredi.substack.com/p/announcing-a-new-project-exploring</t>
+  </si>
+  <si>
+    <t>Roots &amp; Wings by Frank Furedi</t>
+  </si>
+  <si>
+    <t>The Crisis of Competence</t>
+  </si>
+  <si>
+    <t>New project to explore the Crisis of Competence - 1 of the 5 pillars of Anglofuturism</t>
+  </si>
+  <si>
+    <t>Thought provoking, not command to revolution</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -837,6 +950,27 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF1B1814"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFF3EEE4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF5C564C"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color rgb="FF1B1814"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -898,7 +1032,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -930,6 +1064,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1634,7 +1782,7 @@
         <v>153</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>158</v>
@@ -1665,20 +1813,22 @@
         <v>39</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>161</v>
+        <v>247</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>254</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F10" s="6"/>
+        <v>248</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>251</v>
+      </c>
       <c r="G10" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>162</v>
+        <v>249</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>250</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>138</v>
@@ -1699,38 +1849,80 @@
     </row>
     <row r="11" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>255</v>
+      </c>
       <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
+      <c r="G11" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>138</v>
+      </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
+      <c r="M11" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="P11" s="6"/>
     </row>
     <row r="12" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>138</v>
+      </c>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
+      <c r="M12" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="P12" s="6"/>
     </row>
     <row r="13" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -2325,6 +2517,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="H6" r:id="rId1" xr:uid="{277A92A5-EEB4-4955-9C42-F9FC9676B00F}"/>
+    <hyperlink ref="H10" r:id="rId2" xr:uid="{D9DAD9BB-D525-4DEC-8CB1-F3FDD1C93B9D}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -2469,7 +2662,7 @@
         <v>125</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>133</v>
@@ -2500,7 +2693,7 @@
         <v>130</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>132</v>
@@ -2522,22 +2715,22 @@
         <v>39</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="G8" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>169</v>
       </c>
       <c r="I8" s="6">
         <v>7</v>
@@ -2553,22 +2746,22 @@
         <v>39</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>200</v>
-      </c>
       <c r="H9" s="6" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I9" s="6">
         <v>6</v>
@@ -2584,22 +2777,22 @@
         <v>39</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="G10" s="6" t="s">
-        <v>205</v>
-      </c>
       <c r="H10" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="I10" s="6">
         <v>5</v>
@@ -2615,22 +2808,22 @@
         <v>39</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I11" s="6">
         <v>4</v>
@@ -3231,25 +3424,25 @@
         <v>39</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>73</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="H6" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="J6" s="6">
         <v>2012</v>
@@ -3268,25 +3461,25 @@
         <v>39</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>73</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="H7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="I7" s="10" t="s">
         <v>179</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="J7" s="6">
         <v>2004</v>
@@ -3311,19 +3504,19 @@
         <v>73</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="H8" s="10" t="s">
+      <c r="I8" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>186</v>
       </c>
       <c r="J8" s="6">
         <v>1995</v>
@@ -3348,19 +3541,19 @@
         <v>73</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="H9" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="I9" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>191</v>
       </c>
       <c r="J9" s="6">
         <v>2023</v>
@@ -3379,25 +3572,25 @@
         <v>39</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>145</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>211</v>
-      </c>
       <c r="I10" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J10" s="6">
         <v>2026</v>
@@ -3416,25 +3609,25 @@
         <v>39</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>145</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>214</v>
-      </c>
       <c r="I11" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J11" s="6">
         <v>2026</v>
@@ -3453,25 +3646,25 @@
         <v>39</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>145</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>217</v>
-      </c>
       <c r="I12" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="J12" s="6">
         <v>2026</v>
@@ -3490,25 +3683,25 @@
         <v>39</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>145</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="G13" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>223</v>
-      </c>
       <c r="I13" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J13" s="6">
         <v>2026</v>
@@ -3524,28 +3717,28 @@
     <row r="14" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="E14" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="F14" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="G14" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="H14" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>230</v>
-      </c>
       <c r="I14" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="J14" s="6">
         <v>2026</v>
@@ -3564,25 +3757,25 @@
         <v>39</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>145</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J15" s="6">
         <v>2026</v>
@@ -3601,31 +3794,31 @@
         <v>39</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D16" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="G16" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="H16" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>239</v>
-      </c>
       <c r="I16" s="10" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J16" s="6">
         <v>2026</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>49</v>
@@ -4457,4 +4650,440 @@
     <oddFooter>&amp;LNo party mark. No soil-cult.</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F5DF96-B6E5-4036-82B4-1C02651BFAF6}">
+  <sheetPr>
+    <tabColor rgb="FFC9A24A"/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="36" customWidth="1"/>
+    <col min="9" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+    </row>
+    <row r="2" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="M5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="N5" s="15"/>
+    </row>
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I6" s="20">
+        <v>46294</v>
+      </c>
+      <c r="J6" s="20">
+        <v>46308</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" s="10"/>
+    </row>
+    <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="20">
+        <v>46294</v>
+      </c>
+      <c r="J7" s="20">
+        <v>46308</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="N7" s="10"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:N200" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="K5:K200" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>"log,theme-resource,drop"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="D5:D200" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>"essay,video,podcast,substack,paper,other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="B5:B200" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"draft,review,ready,filed,drop"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{114E2E97-9EFE-4C12-8055-2D4DEE7E6DCE}"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ingest five thinkers: Wyvern, Cunliffe, Deutsch, Ridley, FSU
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9954A2F8-9269-4B9D-A92E-B09C305AF7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67DFBA6-59A6-484E-A912-048E81E6C56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="311">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -822,9 +822,6 @@
     <t>Borrow the Aesthetics and convinctions only.</t>
   </si>
   <si>
-    <t>Provides Anglofuturismss core moral aesthetic: the conviction that an authentic future cannot be built on soulless mass-fabrication, but must instead fuse native vernacular craft, organic materials, and human-scale dignity with advanced technological capability.</t>
-  </si>
-  <si>
     <t>show_from</t>
   </si>
   <si>
@@ -892,6 +889,84 @@
   </si>
   <si>
     <t>Thought provoking, not command to revolution</t>
+  </si>
+  <si>
+    <t>The Wyvern Fellowship</t>
+  </si>
+  <si>
+    <t>Preserving Heritage. Building Resilience. Securing our Future.</t>
+  </si>
+  <si>
+    <t>Provides Anglofuturisms core moral aesthetic: the conviction that an authentic future cannot be built on soulless mass-fabrication, but must instead fuse native vernacular craft, organic materials, and human-scale dignity with advanced technological capability.</t>
+  </si>
+  <si>
+    <t>A national fellowship of individuals, families and local chapters working together for mutual support, cultural preservation and community resilience across Britain.</t>
+  </si>
+  <si>
+    <t>Craft, Heritage, Community</t>
+  </si>
+  <si>
+    <t>https://thewyvernfellowship.org.uk/</t>
+  </si>
+  <si>
+    <t>Philip Cunliffe</t>
+  </si>
+  <si>
+    <t>Political theory of Anglofuturism</t>
+  </si>
+  <si>
+    <t>Anglofuturism, Geopolitics</t>
+  </si>
+  <si>
+    <t>https://thephilippics.substack.com/</t>
+  </si>
+  <si>
+    <t>The National Interest bullitin</t>
+  </si>
+  <si>
+    <t>David Deutsch</t>
+  </si>
+  <si>
+    <t>Quantum theory of computation and information</t>
+  </si>
+  <si>
+    <t>Hauling us towards the future one qubit at a time</t>
+  </si>
+  <si>
+    <t>Technologist</t>
+  </si>
+  <si>
+    <t>https://www.daviddeutsch.org.uk/</t>
+  </si>
+  <si>
+    <t>Matt Ridley</t>
+  </si>
+  <si>
+    <t>Innovation</t>
+  </si>
+  <si>
+    <t>The history of innovation blended with rational optimism</t>
+  </si>
+  <si>
+    <t>https://www.rationaloptimistsociety.com/</t>
+  </si>
+  <si>
+    <t>Free Speech Union</t>
+  </si>
+  <si>
+    <t>https://freespeechunion.org/</t>
+  </si>
+  <si>
+    <t>For when you escape the envelope</t>
+  </si>
+  <si>
+    <t>The degrowth antitdote</t>
+  </si>
+  <si>
+    <t>Defenders</t>
+  </si>
+  <si>
+    <t>The guardians of escaping the envelope</t>
   </si>
 </sst>
 </file>
@@ -1058,26 +1133,26 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1392,16 +1467,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="16"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12"/>
+      <c r="B3" s="16"/>
     </row>
     <row r="5" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1519,44 +1594,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
     </row>
     <row r="2" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
     </row>
     <row r="3" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1897,7 +1972,7 @@
         <v>258</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>262</v>
+        <v>287</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>261</v>
@@ -1927,92 +2002,190 @@
     </row>
     <row r="13" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
+      <c r="B13" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>288</v>
+      </c>
       <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="G13" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>138</v>
+      </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
+      <c r="M13" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="P13" s="6"/>
     </row>
     <row r="14" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
+      <c r="B14" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>292</v>
+      </c>
       <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
+      <c r="G14" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>145</v>
+      </c>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
       <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
+      <c r="M14" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O14" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="P14" s="6"/>
     </row>
     <row r="15" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
+      <c r="B15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>298</v>
+      </c>
       <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
+      <c r="G15" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>138</v>
+      </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
+      <c r="M15" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="P15" s="6"/>
     </row>
     <row r="16" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
+      <c r="B16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>308</v>
+      </c>
       <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
+      <c r="G16" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>138</v>
+      </c>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6"/>
+      <c r="M16" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O16" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="P16" s="6"/>
     </row>
     <row r="17" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
+      <c r="B17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>310</v>
+      </c>
       <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
+      <c r="G17" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>138</v>
+      </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
+      <c r="N17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="P17" s="6"/>
     </row>
     <row r="18" spans="1:16" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -2549,34 +2722,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
     </row>
     <row r="3" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -3304,38 +3477,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
     </row>
     <row r="2" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
     </row>
     <row r="3" spans="1:13" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -4293,22 +4466,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -4484,22 +4657,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -4675,124 +4848,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-    </row>
-    <row r="2" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
-        <v>270</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>269</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>263</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>264</v>
-      </c>
-      <c r="K4" s="16" t="s">
+      <c r="D5" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="J5" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="L4" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="N4" s="16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>273</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>267</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>266</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>280</v>
-      </c>
-      <c r="L5" s="15" t="s">
+      <c r="K5" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="L5" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="M5" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="N5" s="15"/>
+      <c r="N5" s="11"/>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
@@ -4800,31 +4973,31 @@
         <v>39</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="F6" s="10" t="s">
+      <c r="G6" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="H6" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="I6" s="14">
+        <v>46294</v>
+      </c>
+      <c r="J6" s="14">
+        <v>46308</v>
+      </c>
+      <c r="K6" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="I6" s="20">
-        <v>46294</v>
-      </c>
-      <c r="J6" s="20">
-        <v>46308</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="L6" s="10" t="s">
         <v>58</v>
@@ -4840,29 +5013,29 @@
         <v>39</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>284</v>
-      </c>
       <c r="H7" s="10"/>
-      <c r="I7" s="20">
+      <c r="I7" s="14">
         <v>46294</v>
       </c>
-      <c r="J7" s="20">
+      <c r="J7" s="14">
         <v>46308</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>192</v>

</xml_diff>

<commit_message>
Ingest Alt-Governance and two Anglofuturism essays
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67DFBA6-59A6-484E-A912-048E81E6C56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D2473A-E67D-40E5-9300-E4082D18BA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="335">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -967,13 +967,85 @@
   </si>
   <si>
     <t>The guardians of escaping the envelope</t>
+  </si>
+  <si>
+    <t>This is Anglofuturism</t>
+  </si>
+  <si>
+    <t>Benjamin De Rebel</t>
+  </si>
+  <si>
+    <t>This is Anglofuturism - The Mallard</t>
+  </si>
+  <si>
+    <t>Anglofuturism: A Primer</t>
+  </si>
+  <si>
+    <t>Early adopter</t>
+  </si>
+  <si>
+    <t>Anglofuturism Digital Trust Network</t>
+  </si>
+  <si>
+    <t>Alfred Atreides</t>
+  </si>
+  <si>
+    <t>https://anglofuturistenthusiast.substack.com/p/digital-serfdom-or-digital-sovereignty</t>
+  </si>
+  <si>
+    <t>The Fight for a Liberty-First Digital Self-Sovereign ID</t>
+  </si>
+  <si>
+    <t>Pro-Technology, Pro-Privacy</t>
+  </si>
+  <si>
+    <t>alt_governance</t>
+  </si>
+  <si>
+    <t>Alt-Governance</t>
+  </si>
+  <si>
+    <t>If there's a new way, I'll be the first in line - it better work this time</t>
+  </si>
+  <si>
+    <t>Evolution, not revolution</t>
+  </si>
+  <si>
+    <t>Emerging shared consciousness across shared thinkers</t>
+  </si>
+  <si>
+    <t>Systems of Governance for the 21st Century</t>
+  </si>
+  <si>
+    <t>Networked Commons Governance</t>
+  </si>
+  <si>
+    <t>Metisocracy</t>
+  </si>
+  <si>
+    <t>https://networkedcommonsgovernance.org/</t>
+  </si>
+  <si>
+    <t>Governance for the Information Age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website </t>
+  </si>
+  <si>
+    <t>The Network State</t>
+  </si>
+  <si>
+    <t>https://thenetworkstate.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balaji Srinivasan </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1050,6 +1122,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF363737"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1107,7 +1186,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1153,6 +1232,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3008,15 +3090,33 @@
     </row>
     <row r="12" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="I12" s="6">
+        <v>3</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -4000,62 +4100,150 @@
     </row>
     <row r="17" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
+      <c r="B17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="J17" s="6">
+        <v>2023</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="M17" s="6"/>
     </row>
     <row r="18" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
+      <c r="B18" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>316</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="J18" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M18" s="6"/>
     </row>
     <row r="19" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="J19" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M19" s="6"/>
     </row>
     <row r="20" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
+      <c r="B20" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="J20" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="M20" s="6"/>
     </row>
     <row r="21" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -4440,6 +4628,10 @@
     <hyperlink ref="G10" r:id="rId2" xr:uid="{DFC55BEA-AE38-403E-9278-B5F569C5550E}"/>
     <hyperlink ref="G14" r:id="rId3" xr:uid="{2A49FE45-E390-45E3-8D17-85E446CE2E31}"/>
     <hyperlink ref="G16" r:id="rId4" xr:uid="{D7BAF8CC-72B4-428E-A765-C89F97972091}"/>
+    <hyperlink ref="G17" r:id="rId5" display="https://mallarduk.com/2023/12/this-is-anglofuturism/" xr:uid="{238D859E-AD6F-4A39-84E1-D0A53819C11E}"/>
+    <hyperlink ref="G18" r:id="rId6" xr:uid="{136CFDDE-0E00-4FAC-B35C-99C411928F3D}"/>
+    <hyperlink ref="G19" r:id="rId7" xr:uid="{DBE3A044-C57A-483B-A614-BE7490D622D8}"/>
+    <hyperlink ref="G20" r:id="rId8" xr:uid="{BDAC1945-5B67-4EFD-A326-C8F4CAB665B2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
File four technology resources: GQI, MIT TR, VentureBeat, Figure
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D2473A-E67D-40E5-9300-E4082D18BA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA14CD69-1FE3-4B4A-913E-73AA704ECA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="355">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -1039,6 +1039,66 @@
   </si>
   <si>
     <t xml:space="preserve">Balaji Srinivasan </t>
+  </si>
+  <si>
+    <t>https://quantumcomputingreport.com/</t>
+  </si>
+  <si>
+    <t>The Quantum Computing Report</t>
+  </si>
+  <si>
+    <t>GQI</t>
+  </si>
+  <si>
+    <t>Don't use this to hack your neighbours wifi router</t>
+  </si>
+  <si>
+    <t>Global Quantum Intelligence</t>
+  </si>
+  <si>
+    <t>https://www.technologyreview.com/</t>
+  </si>
+  <si>
+    <t>MIT Technology Review</t>
+  </si>
+  <si>
+    <t>MIT</t>
+  </si>
+  <si>
+    <t>The future speaks now</t>
+  </si>
+  <si>
+    <t>https://venturebeat.com/</t>
+  </si>
+  <si>
+    <t>The Independent Voice of AI</t>
+  </si>
+  <si>
+    <t>AI Guardians</t>
+  </si>
+  <si>
+    <t>Tracking generative AI, machine learning frameworks, enterprise automation, and autonomous agents from model release to production deployment</t>
+  </si>
+  <si>
+    <t>May include instructions to build a Death Star</t>
+  </si>
+  <si>
+    <t>Observe, orientate, decide, act</t>
+  </si>
+  <si>
+    <t>The future of robotic home help is here</t>
+  </si>
+  <si>
+    <t>Figure AI</t>
+  </si>
+  <si>
+    <t>https://www.figure.ai/</t>
+  </si>
+  <si>
+    <t>The future is much faster than you think</t>
+  </si>
+  <si>
+    <t>Do NOT assemble a droid army</t>
   </si>
 </sst>
 </file>
@@ -1222,19 +1282,19 @@
     <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1549,16 +1609,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="17"/>
     </row>
     <row r="5" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1676,44 +1736,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
     </row>
     <row r="2" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
     </row>
     <row r="3" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2804,34 +2864,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -3577,38 +3637,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
     </row>
     <row r="2" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
     </row>
     <row r="3" spans="1:13" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -4146,7 +4206,7 @@
       <c r="D18" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="E18" s="21" t="s">
+      <c r="E18" s="15" t="s">
         <v>316</v>
       </c>
       <c r="F18" s="10" t="s">
@@ -4248,62 +4308,150 @@
     </row>
     <row r="21" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
+      <c r="B21" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="J21" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="M21" s="6"/>
     </row>
     <row r="22" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
+      <c r="B22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="J22" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="M22" s="6"/>
     </row>
     <row r="23" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
+      <c r="B23" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="J23" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="M23" s="6"/>
     </row>
     <row r="24" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
+      <c r="B24" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J24" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="M24" s="6"/>
     </row>
     <row r="25" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -4632,6 +4780,10 @@
     <hyperlink ref="G18" r:id="rId6" xr:uid="{136CFDDE-0E00-4FAC-B35C-99C411928F3D}"/>
     <hyperlink ref="G19" r:id="rId7" xr:uid="{DBE3A044-C57A-483B-A614-BE7490D622D8}"/>
     <hyperlink ref="G20" r:id="rId8" xr:uid="{BDAC1945-5B67-4EFD-A326-C8F4CAB665B2}"/>
+    <hyperlink ref="G21" r:id="rId9" xr:uid="{21513DE6-CF36-4152-A0B9-AA7BFFA71FE5}"/>
+    <hyperlink ref="G22" r:id="rId10" xr:uid="{B79DAC40-5B86-4FA8-B176-C84821294AC2}"/>
+    <hyperlink ref="G23" r:id="rId11" xr:uid="{FE3FBEA6-ACDD-40EE-843C-E57AEC643A63}"/>
+    <hyperlink ref="G24" r:id="rId12" xr:uid="{B9402A62-A230-41F8-96EE-C6D4732CBA20}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -4658,22 +4810,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -4849,22 +5001,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5040,40 +5192,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
     </row>
     <row r="2" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">

</xml_diff>

<commit_message>
Roll intercepts to 13–27 Oct window
</commit_message>
<xml_diff>
--- a/content/open-sky-catalog.xlsx
+++ b/content/open-sky-catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Anglofuturism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA14CD69-1FE3-4B4A-913E-73AA704ECA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF52D748-9751-4601-91C6-A1777ED18C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HOW" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="369">
   <si>
     <t>OPEN SKY — content catalog</t>
   </si>
@@ -1099,6 +1099,48 @@
   </si>
   <si>
     <t>Do NOT assemble a droid army</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=LRdb8UmPnh0</t>
+  </si>
+  <si>
+    <t>video</t>
+  </si>
+  <si>
+    <t>The Coming Manhattan Project</t>
+  </si>
+  <si>
+    <t>Peter H. Diamandis</t>
+  </si>
+  <si>
+    <t>AI's 1942 moment</t>
+  </si>
+  <si>
+    <t>Don't fear the future</t>
+  </si>
+  <si>
+    <t>https://podcasts.apple.com/gb/podcast/rodolfo-rosini-ceo-vaire-computing-is-building-ai-chips/id1743404902?i=1000793208069</t>
+  </si>
+  <si>
+    <t>The future of computing has to run in reverse.</t>
+  </si>
+  <si>
+    <t>https://substack.com/home/post/p-196794597</t>
+  </si>
+  <si>
+    <t>Welcome to Proto-Town</t>
+  </si>
+  <si>
+    <t>The Rational Optimist</t>
+  </si>
+  <si>
+    <t>Escape the bureaucracy and build</t>
+  </si>
+  <si>
+    <t>alt-governance</t>
+  </si>
+  <si>
+    <t>Front running the compute crunch</t>
   </si>
 </sst>
 </file>
@@ -1285,16 +1327,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1609,7 +1651,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="17"/>
@@ -1736,7 +1778,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="17"/>
@@ -1756,7 +1798,7 @@
       <c r="P1" s="17"/>
     </row>
     <row r="2" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="17"/>
@@ -2864,7 +2906,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B1" s="17"/>
@@ -2879,7 +2921,7 @@
       <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="17"/>
@@ -3637,7 +3679,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="17"/>
@@ -3654,7 +3696,7 @@
       <c r="M1" s="17"/>
     </row>
     <row r="2" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>66</v>
       </c>
       <c r="B2" s="17"/>
@@ -4810,7 +4852,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>81</v>
       </c>
       <c r="B1" s="17"/>
@@ -4819,7 +4861,7 @@
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="17"/>
@@ -5001,7 +5043,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>101</v>
       </c>
       <c r="B1" s="17"/>
@@ -5010,7 +5052,7 @@
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>102</v>
       </c>
       <c r="B2" s="17"/>
@@ -5192,7 +5234,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="18" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="17"/>
@@ -5210,7 +5252,7 @@
       <c r="N1" s="17"/>
     </row>
     <row r="2" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="16" t="s">
         <v>269</v>
       </c>
       <c r="B2" s="17"/>
@@ -5389,52 +5431,120 @@
       </c>
       <c r="N7" s="10"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
+      <c r="B8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="I8" s="14">
+        <v>46308</v>
+      </c>
+      <c r="J8" s="14">
+        <v>46322</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="N8" s="10"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>368</v>
+      </c>
       <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
+      <c r="I9" s="14">
+        <v>46308</v>
+      </c>
+      <c r="J9" s="14">
+        <v>46322</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="N9" s="10"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="B10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>366</v>
+      </c>
       <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
+      <c r="I10" s="14">
+        <v>46308</v>
+      </c>
+      <c r="J10" s="14">
+        <v>46322</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>49</v>
+      </c>
       <c r="N10" s="10"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>